<commit_message>
calculation of new indicators
</commit_message>
<xml_diff>
--- a/scheme/Cadastro/issues_metadados_cadastro.xlsx
+++ b/scheme/Cadastro/issues_metadados_cadastro.xlsx
@@ -65394,7 +65394,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MQMS01</t>
+          <t>MQME001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -65409,7 +65409,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MQMS02</t>
+          <t>MQME002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -65424,7 +65424,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MQMS03</t>
+          <t>MQME003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -65439,7 +65439,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MQMS04</t>
+          <t>MQME004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -65454,7 +65454,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MQMS05</t>
+          <t>MQME005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -65525,7 +65525,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MQME10</t>
+          <t>MQME012</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -65551,7 +65551,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -65581,7 +65581,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -65611,7 +65611,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -65641,7 +65641,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -65671,7 +65671,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -65701,7 +65701,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -65731,7 +65731,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -65761,7 +65761,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -65791,7 +65791,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -65821,7 +65821,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -65851,7 +65851,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -65881,7 +65881,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -65911,7 +65911,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -65941,7 +65941,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -65971,7 +65971,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -66001,7 +66001,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -66031,7 +66031,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -66061,7 +66061,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -66091,7 +66091,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -66121,7 +66121,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -66151,7 +66151,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -66181,7 +66181,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -66211,7 +66211,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -66241,7 +66241,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -66271,7 +66271,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -66301,7 +66301,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -66331,7 +66331,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -66361,7 +66361,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -66391,7 +66391,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -66421,7 +66421,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -66451,7 +66451,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -66481,7 +66481,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -66511,7 +66511,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -66541,7 +66541,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -66571,7 +66571,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -66601,7 +66601,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -66631,7 +66631,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -66661,7 +66661,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -66691,7 +66691,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -66721,7 +66721,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -66751,7 +66751,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -66781,7 +66781,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -66811,7 +66811,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -66841,7 +66841,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -66871,7 +66871,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -66901,7 +66901,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -66931,7 +66931,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -66961,7 +66961,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -66991,7 +66991,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -67021,7 +67021,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -67051,7 +67051,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -67081,7 +67081,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -67111,7 +67111,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -67141,7 +67141,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -67171,7 +67171,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -67201,7 +67201,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -67231,7 +67231,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -67261,7 +67261,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -67291,7 +67291,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -67321,7 +67321,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -67351,7 +67351,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -67381,7 +67381,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -67411,7 +67411,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -67441,7 +67441,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -67471,7 +67471,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -67501,7 +67501,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -67531,7 +67531,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -67561,7 +67561,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -67591,7 +67591,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -67621,7 +67621,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -67651,7 +67651,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -67681,7 +67681,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -67711,7 +67711,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -67741,7 +67741,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -67771,7 +67771,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -67801,7 +67801,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -67831,7 +67831,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -67861,7 +67861,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -67891,7 +67891,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -67921,7 +67921,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -67951,7 +67951,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -67981,7 +67981,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -68011,7 +68011,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -68041,7 +68041,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -68071,7 +68071,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -68101,7 +68101,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -68131,7 +68131,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -68161,7 +68161,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -68191,7 +68191,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -68221,7 +68221,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -68251,7 +68251,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -68281,7 +68281,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>MQME12</t>
+          <t>MQME014</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -68311,7 +68311,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -68341,7 +68341,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -68371,7 +68371,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -68401,7 +68401,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -68431,7 +68431,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -68461,7 +68461,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -68491,7 +68491,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -68521,7 +68521,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -68551,7 +68551,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -68581,7 +68581,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -68611,7 +68611,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -68641,7 +68641,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -68671,7 +68671,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -68701,7 +68701,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -68731,7 +68731,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -68761,7 +68761,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -68791,7 +68791,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -68821,7 +68821,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -68851,7 +68851,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -68881,7 +68881,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -68911,7 +68911,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -68941,7 +68941,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -68971,7 +68971,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -69001,7 +69001,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -69031,7 +69031,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -69061,7 +69061,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -69091,7 +69091,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -69121,7 +69121,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -69151,7 +69151,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -69181,7 +69181,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -69211,7 +69211,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -69241,7 +69241,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -69271,7 +69271,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -69301,7 +69301,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -69331,7 +69331,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -69361,7 +69361,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -69391,7 +69391,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -69421,7 +69421,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -69451,7 +69451,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -69481,7 +69481,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -69511,7 +69511,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -69541,7 +69541,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -69571,7 +69571,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -69601,7 +69601,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -69631,7 +69631,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -69661,7 +69661,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -69691,7 +69691,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -69721,7 +69721,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -69751,7 +69751,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -69781,7 +69781,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -69811,7 +69811,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -69841,7 +69841,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -69871,7 +69871,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -69901,7 +69901,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -69931,7 +69931,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -69961,7 +69961,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -69991,7 +69991,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -70021,7 +70021,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -70051,7 +70051,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -70081,7 +70081,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -70111,7 +70111,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -70141,7 +70141,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -70171,7 +70171,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -70201,7 +70201,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -70231,7 +70231,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -70261,7 +70261,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -70291,7 +70291,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -70321,7 +70321,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -70351,7 +70351,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -70381,7 +70381,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -70411,7 +70411,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -70441,7 +70441,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -70471,7 +70471,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -70501,7 +70501,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -70531,7 +70531,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -70561,7 +70561,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -70591,7 +70591,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -70621,7 +70621,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -70651,7 +70651,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -70681,7 +70681,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -70711,7 +70711,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -70741,7 +70741,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -70771,7 +70771,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -70801,7 +70801,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -70831,7 +70831,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -70861,7 +70861,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -70891,7 +70891,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -70921,7 +70921,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -70951,7 +70951,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -70981,7 +70981,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -71011,7 +71011,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -71041,7 +71041,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -71071,7 +71071,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -71101,7 +71101,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -71131,7 +71131,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -71161,7 +71161,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -71191,7 +71191,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -71221,7 +71221,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -71251,7 +71251,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -71281,7 +71281,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -71311,7 +71311,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -71341,7 +71341,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -71371,7 +71371,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -71401,7 +71401,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -71431,7 +71431,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -71461,7 +71461,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -71491,7 +71491,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -71521,7 +71521,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -71551,7 +71551,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -71581,7 +71581,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -71611,7 +71611,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -71641,7 +71641,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -71671,7 +71671,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -71701,7 +71701,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -71731,7 +71731,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -71761,7 +71761,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -71791,7 +71791,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -71821,7 +71821,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -71851,7 +71851,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -71881,7 +71881,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -71911,7 +71911,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -71941,7 +71941,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -71971,7 +71971,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -72001,7 +72001,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -72031,7 +72031,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -72061,7 +72061,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -72091,7 +72091,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -72121,7 +72121,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -72151,7 +72151,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -72181,7 +72181,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -72211,7 +72211,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -72241,7 +72241,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -72271,7 +72271,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -72301,7 +72301,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -72331,7 +72331,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -72361,7 +72361,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -72391,7 +72391,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -72421,7 +72421,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -72451,7 +72451,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -72481,7 +72481,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -72511,7 +72511,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -72541,7 +72541,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -72571,7 +72571,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -72601,7 +72601,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -72631,7 +72631,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -72661,7 +72661,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -72691,7 +72691,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -72721,7 +72721,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -72751,7 +72751,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -72781,7 +72781,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -72811,7 +72811,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -72841,7 +72841,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -72871,7 +72871,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -72901,7 +72901,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -72931,7 +72931,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -72961,7 +72961,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -72991,7 +72991,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -73021,7 +73021,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -73051,7 +73051,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -73081,7 +73081,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -73111,7 +73111,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -73141,7 +73141,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -73171,7 +73171,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -73201,7 +73201,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -73231,7 +73231,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -73261,7 +73261,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -73291,7 +73291,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
@@ -73321,7 +73321,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -73351,7 +73351,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
@@ -73381,7 +73381,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -73411,7 +73411,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -73441,7 +73441,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -73471,7 +73471,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -73501,7 +73501,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -73531,7 +73531,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -73561,7 +73561,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -73591,7 +73591,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -73621,7 +73621,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -73651,7 +73651,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -73681,7 +73681,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
@@ -73711,7 +73711,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -73741,7 +73741,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
@@ -73771,7 +73771,7 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
@@ -73801,7 +73801,7 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
@@ -73831,7 +73831,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
@@ -73861,7 +73861,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
@@ -73891,7 +73891,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
@@ -73921,7 +73921,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
@@ -73951,7 +73951,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
@@ -73981,7 +73981,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
@@ -74011,7 +74011,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
@@ -74041,7 +74041,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
@@ -74071,7 +74071,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
@@ -74101,7 +74101,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
@@ -74131,7 +74131,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
@@ -74161,7 +74161,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
@@ -74191,7 +74191,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
@@ -74221,7 +74221,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
@@ -74251,7 +74251,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -74281,7 +74281,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -74311,7 +74311,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -74341,7 +74341,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -74371,7 +74371,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
@@ -74401,7 +74401,7 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
@@ -74431,7 +74431,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
@@ -74461,7 +74461,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
@@ -74491,7 +74491,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
@@ -74521,7 +74521,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
@@ -74551,7 +74551,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
@@ -74581,7 +74581,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
@@ -74611,7 +74611,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -74641,7 +74641,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
@@ -74671,7 +74671,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
@@ -74701,7 +74701,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
@@ -74731,7 +74731,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
@@ -74761,7 +74761,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
@@ -74791,7 +74791,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
@@ -74821,7 +74821,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
@@ -74851,7 +74851,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
@@ -74881,7 +74881,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
@@ -74911,7 +74911,7 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
@@ -74941,7 +74941,7 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
@@ -74971,7 +74971,7 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
@@ -75001,7 +75001,7 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
@@ -75031,7 +75031,7 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
@@ -75061,7 +75061,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
@@ -75091,7 +75091,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
@@ -75121,7 +75121,7 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
@@ -75151,7 +75151,7 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
@@ -75181,7 +75181,7 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
@@ -75211,7 +75211,7 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
@@ -75241,7 +75241,7 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
@@ -75271,7 +75271,7 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
@@ -75301,7 +75301,7 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
@@ -75331,7 +75331,7 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
@@ -75361,7 +75361,7 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
@@ -75391,7 +75391,7 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
@@ -75421,7 +75421,7 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
@@ -75451,7 +75451,7 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
@@ -75481,7 +75481,7 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
@@ -75511,7 +75511,7 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
@@ -75541,7 +75541,7 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
@@ -75571,7 +75571,7 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
@@ -75601,7 +75601,7 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
@@ -75631,7 +75631,7 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
@@ -75661,7 +75661,7 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
@@ -75691,7 +75691,7 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
@@ -75721,7 +75721,7 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
@@ -75751,7 +75751,7 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
@@ -75781,7 +75781,7 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
@@ -75811,7 +75811,7 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
@@ -75841,7 +75841,7 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
@@ -75871,7 +75871,7 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
@@ -75901,7 +75901,7 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
@@ -75931,7 +75931,7 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
@@ -75961,7 +75961,7 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
@@ -75991,7 +75991,7 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
@@ -76021,7 +76021,7 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
@@ -76051,7 +76051,7 @@
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
@@ -76081,7 +76081,7 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
@@ -76111,7 +76111,7 @@
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
@@ -76141,7 +76141,7 @@
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
@@ -76171,7 +76171,7 @@
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
@@ -76201,7 +76201,7 @@
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
@@ -76231,7 +76231,7 @@
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
@@ -76261,7 +76261,7 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
@@ -76291,7 +76291,7 @@
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
@@ -76321,7 +76321,7 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
@@ -76351,7 +76351,7 @@
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
@@ -76381,7 +76381,7 @@
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
@@ -76411,7 +76411,7 @@
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
@@ -76441,7 +76441,7 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
@@ -76471,7 +76471,7 @@
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
@@ -76501,7 +76501,7 @@
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
@@ -76531,7 +76531,7 @@
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
@@ -76561,7 +76561,7 @@
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
@@ -76591,7 +76591,7 @@
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
@@ -76621,7 +76621,7 @@
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
@@ -76651,7 +76651,7 @@
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
@@ -76681,7 +76681,7 @@
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
@@ -76711,7 +76711,7 @@
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
@@ -76741,7 +76741,7 @@
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
@@ -76771,7 +76771,7 @@
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
@@ -76801,7 +76801,7 @@
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B378" t="inlineStr">
@@ -76831,7 +76831,7 @@
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B379" t="inlineStr">
@@ -76861,7 +76861,7 @@
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B380" t="inlineStr">
@@ -76891,7 +76891,7 @@
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B381" t="inlineStr">
@@ -76921,7 +76921,7 @@
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B382" t="inlineStr">
@@ -76951,7 +76951,7 @@
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B383" t="inlineStr">
@@ -76981,7 +76981,7 @@
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B384" t="inlineStr">
@@ -77011,7 +77011,7 @@
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B385" t="inlineStr">
@@ -77041,7 +77041,7 @@
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B386" t="inlineStr">
@@ -77071,7 +77071,7 @@
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B387" t="inlineStr">
@@ -77101,7 +77101,7 @@
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
@@ -77131,7 +77131,7 @@
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
@@ -77161,7 +77161,7 @@
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B390" t="inlineStr">
@@ -77191,7 +77191,7 @@
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B391" t="inlineStr">
@@ -77221,7 +77221,7 @@
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
@@ -77251,7 +77251,7 @@
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
@@ -77281,7 +77281,7 @@
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B394" t="inlineStr">
@@ -77311,7 +77311,7 @@
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B395" t="inlineStr">
@@ -77341,7 +77341,7 @@
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B396" t="inlineStr">
@@ -77371,7 +77371,7 @@
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B397" t="inlineStr">
@@ -77401,7 +77401,7 @@
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
@@ -77431,7 +77431,7 @@
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
@@ -77461,7 +77461,7 @@
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
@@ -77491,7 +77491,7 @@
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B401" t="inlineStr">
@@ -77521,7 +77521,7 @@
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B402" t="inlineStr">
@@ -77551,7 +77551,7 @@
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B403" t="inlineStr">
@@ -77581,7 +77581,7 @@
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B404" t="inlineStr">
@@ -77611,7 +77611,7 @@
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B405" t="inlineStr">
@@ -77641,7 +77641,7 @@
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B406" t="inlineStr">
@@ -77671,7 +77671,7 @@
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
@@ -77701,7 +77701,7 @@
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
@@ -77731,7 +77731,7 @@
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B409" t="inlineStr">
@@ -77761,7 +77761,7 @@
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B410" t="inlineStr">
@@ -77791,7 +77791,7 @@
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B411" t="inlineStr">
@@ -77821,7 +77821,7 @@
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
@@ -77851,7 +77851,7 @@
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
@@ -77881,7 +77881,7 @@
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B414" t="inlineStr">
@@ -77911,7 +77911,7 @@
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B415" t="inlineStr">
@@ -77941,7 +77941,7 @@
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B416" t="inlineStr">
@@ -77971,7 +77971,7 @@
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B417" t="inlineStr">
@@ -78001,7 +78001,7 @@
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B418" t="inlineStr">
@@ -78031,7 +78031,7 @@
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B419" t="inlineStr">
@@ -78061,7 +78061,7 @@
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B420" t="inlineStr">
@@ -78091,7 +78091,7 @@
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B421" t="inlineStr">
@@ -78121,7 +78121,7 @@
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B422" t="inlineStr">
@@ -78151,7 +78151,7 @@
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B423" t="inlineStr">
@@ -78181,7 +78181,7 @@
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B424" t="inlineStr">
@@ -78211,7 +78211,7 @@
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B425" t="inlineStr">
@@ -78241,7 +78241,7 @@
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B426" t="inlineStr">
@@ -78271,7 +78271,7 @@
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B427" t="inlineStr">
@@ -78301,7 +78301,7 @@
     <row r="428">
       <c r="A428" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B428" t="inlineStr">
@@ -78331,7 +78331,7 @@
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B429" t="inlineStr">
@@ -78361,7 +78361,7 @@
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B430" t="inlineStr">
@@ -78391,7 +78391,7 @@
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B431" t="inlineStr">
@@ -78421,7 +78421,7 @@
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B432" t="inlineStr">
@@ -78451,7 +78451,7 @@
     <row r="433">
       <c r="A433" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B433" t="inlineStr">
@@ -78481,7 +78481,7 @@
     <row r="434">
       <c r="A434" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B434" t="inlineStr">
@@ -78511,7 +78511,7 @@
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
@@ -78541,7 +78541,7 @@
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B436" t="inlineStr">
@@ -78571,7 +78571,7 @@
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B437" t="inlineStr">
@@ -78601,7 +78601,7 @@
     <row r="438">
       <c r="A438" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B438" t="inlineStr">
@@ -78631,7 +78631,7 @@
     <row r="439">
       <c r="A439" t="inlineStr">
         <is>
-          <t>MQME01</t>
+          <t>MQME008</t>
         </is>
       </c>
       <c r="B439" t="inlineStr">
@@ -78661,7 +78661,7 @@
     <row r="440">
       <c r="A440" t="inlineStr">
         <is>
-          <t>MQME14</t>
+          <t>MQME009</t>
         </is>
       </c>
       <c r="B440" t="inlineStr">
@@ -78695,7 +78695,7 @@
     <row r="441">
       <c r="A441" t="inlineStr">
         <is>
-          <t>MQME14</t>
+          <t>MQME009</t>
         </is>
       </c>
       <c r="B441" t="inlineStr">
@@ -78729,7 +78729,7 @@
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>MQME14</t>
+          <t>MQME009</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
@@ -78763,7 +78763,7 @@
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>MQME14</t>
+          <t>MQME009</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
@@ -78797,7 +78797,7 @@
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>MQME14</t>
+          <t>MQME009</t>
         </is>
       </c>
       <c r="B444" t="inlineStr">
@@ -78831,7 +78831,7 @@
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>MQME14</t>
+          <t>MQME009</t>
         </is>
       </c>
       <c r="B445" t="inlineStr">
@@ -78865,7 +78865,7 @@
     <row r="446">
       <c r="A446" t="inlineStr">
         <is>
-          <t>MQME14</t>
+          <t>MQME009</t>
         </is>
       </c>
       <c r="B446" t="inlineStr">
@@ -78899,7 +78899,7 @@
     <row r="447">
       <c r="A447" t="inlineStr">
         <is>
-          <t>MQME14</t>
+          <t>MQME009</t>
         </is>
       </c>
       <c r="B447" t="inlineStr">
@@ -78933,7 +78933,7 @@
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t>MQME14</t>
+          <t>MQME009</t>
         </is>
       </c>
       <c r="B448" t="inlineStr">
@@ -78967,7 +78967,7 @@
     <row r="449">
       <c r="A449" t="inlineStr">
         <is>
-          <t>MQME14</t>
+          <t>MQME009</t>
         </is>
       </c>
       <c r="B449" t="inlineStr">
@@ -79001,7 +79001,7 @@
     <row r="450">
       <c r="A450" t="inlineStr">
         <is>
-          <t>MQME14</t>
+          <t>MQME009</t>
         </is>
       </c>
       <c r="B450" t="inlineStr">
@@ -79035,7 +79035,7 @@
     <row r="451">
       <c r="A451" t="inlineStr">
         <is>
-          <t>MQME14</t>
+          <t>MQME009</t>
         </is>
       </c>
       <c r="B451" t="inlineStr">
@@ -79069,7 +79069,7 @@
     <row r="452">
       <c r="A452" t="inlineStr">
         <is>
-          <t>MQME14</t>
+          <t>MQME009</t>
         </is>
       </c>
       <c r="B452" t="inlineStr">
@@ -79103,7 +79103,7 @@
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t>MQME14</t>
+          <t>MQME009</t>
         </is>
       </c>
       <c r="B453" t="inlineStr">
@@ -79137,7 +79137,7 @@
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t>MQME14</t>
+          <t>MQME009</t>
         </is>
       </c>
       <c r="B454" t="inlineStr">
@@ -79171,7 +79171,7 @@
     <row r="455">
       <c r="A455" t="inlineStr">
         <is>
-          <t>MQME14</t>
+          <t>MQME009</t>
         </is>
       </c>
       <c r="B455" t="inlineStr">
@@ -79205,7 +79205,7 @@
     <row r="456">
       <c r="A456" t="inlineStr">
         <is>
-          <t>MQME14</t>
+          <t>MQME009</t>
         </is>
       </c>
       <c r="B456" t="inlineStr">
@@ -79239,7 +79239,7 @@
     <row r="457">
       <c r="A457" t="inlineStr">
         <is>
-          <t>MQME14</t>
+          <t>MQME009</t>
         </is>
       </c>
       <c r="B457" t="inlineStr">
@@ -79273,7 +79273,7 @@
     <row r="458">
       <c r="A458" t="inlineStr">
         <is>
-          <t>MQME14</t>
+          <t>MQME009</t>
         </is>
       </c>
       <c r="B458" t="inlineStr">
@@ -79307,7 +79307,7 @@
     <row r="459">
       <c r="A459" t="inlineStr">
         <is>
-          <t>MQME14</t>
+          <t>MQME009</t>
         </is>
       </c>
       <c r="B459" t="inlineStr">
@@ -79341,7 +79341,7 @@
     <row r="460">
       <c r="A460" t="inlineStr">
         <is>
-          <t>MQME14</t>
+          <t>MQME009</t>
         </is>
       </c>
       <c r="B460" t="inlineStr">
@@ -79375,7 +79375,7 @@
     <row r="461">
       <c r="A461" t="inlineStr">
         <is>
-          <t>MQME14</t>
+          <t>MQME009</t>
         </is>
       </c>
       <c r="B461" t="inlineStr">
@@ -79409,7 +79409,7 @@
     <row r="462">
       <c r="A462" t="inlineStr">
         <is>
-          <t>MQME14</t>
+          <t>MQME009</t>
         </is>
       </c>
       <c r="B462" t="inlineStr">
@@ -79443,7 +79443,7 @@
     <row r="463">
       <c r="A463" t="inlineStr">
         <is>
-          <t>MQME14</t>
+          <t>MQME009</t>
         </is>
       </c>
       <c r="B463" t="inlineStr">
@@ -79477,7 +79477,7 @@
     <row r="464">
       <c r="A464" t="inlineStr">
         <is>
-          <t>MQME14</t>
+          <t>MQME009</t>
         </is>
       </c>
       <c r="B464" t="inlineStr">
@@ -79511,7 +79511,7 @@
     <row r="465">
       <c r="A465" t="inlineStr">
         <is>
-          <t>MQME15</t>
+          <t>MQME010</t>
         </is>
       </c>
       <c r="B465" t="inlineStr">
@@ -79545,7 +79545,7 @@
     <row r="466">
       <c r="A466" t="inlineStr">
         <is>
-          <t>MQME15</t>
+          <t>MQME010</t>
         </is>
       </c>
       <c r="B466" t="inlineStr">
@@ -79579,7 +79579,7 @@
     <row r="467">
       <c r="A467" t="inlineStr">
         <is>
-          <t>MQME15</t>
+          <t>MQME010</t>
         </is>
       </c>
       <c r="B467" t="inlineStr">
@@ -79613,7 +79613,7 @@
     <row r="468">
       <c r="A468" t="inlineStr">
         <is>
-          <t>MQME15</t>
+          <t>MQME010</t>
         </is>
       </c>
       <c r="B468" t="inlineStr">
@@ -79647,7 +79647,7 @@
     <row r="469">
       <c r="A469" t="inlineStr">
         <is>
-          <t>MQME15</t>
+          <t>MQME010</t>
         </is>
       </c>
       <c r="B469" t="inlineStr">
@@ -79681,7 +79681,7 @@
     <row r="470">
       <c r="A470" t="inlineStr">
         <is>
-          <t>MQME15</t>
+          <t>MQME010</t>
         </is>
       </c>
       <c r="B470" t="inlineStr">
@@ -79715,7 +79715,7 @@
     <row r="471">
       <c r="A471" t="inlineStr">
         <is>
-          <t>MQME15</t>
+          <t>MQME010</t>
         </is>
       </c>
       <c r="B471" t="inlineStr">
@@ -79749,7 +79749,7 @@
     <row r="472">
       <c r="A472" t="inlineStr">
         <is>
-          <t>MQME15</t>
+          <t>MQME010</t>
         </is>
       </c>
       <c r="B472" t="inlineStr">
@@ -79783,7 +79783,7 @@
     <row r="473">
       <c r="A473" t="inlineStr">
         <is>
-          <t>MQME15</t>
+          <t>MQME010</t>
         </is>
       </c>
       <c r="B473" t="inlineStr">
@@ -79817,7 +79817,7 @@
     <row r="474">
       <c r="A474" t="inlineStr">
         <is>
-          <t>MQME15</t>
+          <t>MQME010</t>
         </is>
       </c>
       <c r="B474" t="inlineStr">
@@ -79851,7 +79851,7 @@
     <row r="475">
       <c r="A475" t="inlineStr">
         <is>
-          <t>MQME15</t>
+          <t>MQME010</t>
         </is>
       </c>
       <c r="B475" t="inlineStr">
@@ -79885,7 +79885,7 @@
     <row r="476">
       <c r="A476" t="inlineStr">
         <is>
-          <t>MQME15</t>
+          <t>MQME010</t>
         </is>
       </c>
       <c r="B476" t="inlineStr">
@@ -79919,7 +79919,7 @@
     <row r="477">
       <c r="A477" t="inlineStr">
         <is>
-          <t>MQME15</t>
+          <t>MQME010</t>
         </is>
       </c>
       <c r="B477" t="inlineStr">
@@ -79953,7 +79953,7 @@
     <row r="478">
       <c r="A478" t="inlineStr">
         <is>
-          <t>MQME15</t>
+          <t>MQME010</t>
         </is>
       </c>
       <c r="B478" t="inlineStr">
@@ -79987,7 +79987,7 @@
     <row r="479">
       <c r="A479" t="inlineStr">
         <is>
-          <t>MQME15</t>
+          <t>MQME010</t>
         </is>
       </c>
       <c r="B479" t="inlineStr">
@@ -80021,7 +80021,7 @@
     <row r="480">
       <c r="A480" t="inlineStr">
         <is>
-          <t>MQME15</t>
+          <t>MQME010</t>
         </is>
       </c>
       <c r="B480" t="inlineStr">
@@ -80055,7 +80055,7 @@
     <row r="481">
       <c r="A481" t="inlineStr">
         <is>
-          <t>MQME15</t>
+          <t>MQME010</t>
         </is>
       </c>
       <c r="B481" t="inlineStr">
@@ -80089,7 +80089,7 @@
     <row r="482">
       <c r="A482" t="inlineStr">
         <is>
-          <t>MQME15</t>
+          <t>MQME010</t>
         </is>
       </c>
       <c r="B482" t="inlineStr">
@@ -80123,7 +80123,7 @@
     <row r="483">
       <c r="A483" t="inlineStr">
         <is>
-          <t>MQME15</t>
+          <t>MQME010</t>
         </is>
       </c>
       <c r="B483" t="inlineStr">
@@ -80157,7 +80157,7 @@
     <row r="484">
       <c r="A484" t="inlineStr">
         <is>
-          <t>MQME15</t>
+          <t>MQME010</t>
         </is>
       </c>
       <c r="B484" t="inlineStr">
@@ -80191,7 +80191,7 @@
     <row r="485">
       <c r="A485" t="inlineStr">
         <is>
-          <t>MQME15</t>
+          <t>MQME010</t>
         </is>
       </c>
       <c r="B485" t="inlineStr">
@@ -80225,7 +80225,7 @@
     <row r="486">
       <c r="A486" t="inlineStr">
         <is>
-          <t>MQME15</t>
+          <t>MQME010</t>
         </is>
       </c>
       <c r="B486" t="inlineStr">
@@ -80259,7 +80259,7 @@
     <row r="487">
       <c r="A487" t="inlineStr">
         <is>
-          <t>MQME15</t>
+          <t>MQME010</t>
         </is>
       </c>
       <c r="B487" t="inlineStr">
@@ -80293,7 +80293,7 @@
     <row r="488">
       <c r="A488" t="inlineStr">
         <is>
-          <t>MQME15</t>
+          <t>MQME010</t>
         </is>
       </c>
       <c r="B488" t="inlineStr">
@@ -80327,7 +80327,7 @@
     <row r="489">
       <c r="A489" t="inlineStr">
         <is>
-          <t>MQME15</t>
+          <t>MQME010</t>
         </is>
       </c>
       <c r="B489" t="inlineStr">
@@ -80361,7 +80361,7 @@
     <row r="490">
       <c r="A490" t="inlineStr">
         <is>
-          <t>MQME15</t>
+          <t>MQME010</t>
         </is>
       </c>
       <c r="B490" t="inlineStr">
@@ -80403,7 +80403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -80426,45 +80426,30 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MQME00</t>
+          <t>MQME006</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Total number of columns</t>
+          <t>Total number of length-required columns</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1042</v>
+        <v>423</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MQMEA1</t>
+          <t>MQME007</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Total number of length-required columns</t>
+          <t>Total number of NUMBER columns</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>MQMEA2</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Total number of NUMBER columns</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
         <v>476</v>
       </c>
     </row>
@@ -80479,7 +80464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -80502,29 +80487,29 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>IQME01</t>
+          <t>MQID001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Columns with comments</t>
+          <t>Table names in singular</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>66.89%</t>
+          <t>98.89%</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>IQME02</t>
+          <t>MQID002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Columns with data type</t>
+          <t>Table with recommended name length</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -80536,29 +80521,29 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>IQME03</t>
+          <t>MQID003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Length-required columns with data length</t>
+          <t>Columns with correct prefixes</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>91.17%</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>IQME04</t>
+          <t>MQID004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>NUMBER columns with valid scale</t>
+          <t>Columns with recommended name size</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -80570,49 +80555,117 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>IQME05</t>
+          <t>MQID005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Columns with valid num_distinct</t>
+          <t>Columns with comments</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>66.89%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>IQME06</t>
+          <t>MQID006</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Columns with valid num_nulls</t>
+          <t>Table with standard PK prefixes</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>64.79%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>IQME07</t>
+          <t>MQID007</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Columns with valid density</t>
+          <t>Table with standard FK prefixes</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
+        <is>
+          <t>61.19%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MQID008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Table with standard UK prefixes</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MQID009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>NUMBER columns with valid scale</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>MQID010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Columns with valid num_distinct</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>MQID011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Columns with valid num_nulls</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
         <is>
           <t>100.00%</t>
         </is>

</xml_diff>